<commit_message>
Herzie demodata en verwijder ongebruikte 1CHO-kolommen
demo Leiden is nu een masterselectie Farmacie die de structuur van de
FAR Leiden 2025-dummy volgt (enkele kop-rij, beoordelaars B1/B2,
puntenscores per onderdeel, diploma als uitkomst). demo Radboud blijft de
Psychologie-bachelorstructuur. Zo lijken de twee demo's niet langer op
elkaar.

herkomst en gem_eindcijfer_vo worden nergens meer getoond (de VO-tab is
verdwenen, demografie gebruikt alleen geslacht en vooropleiding), dus die
passthrough-kolommen zijn uit cho_transform, de datascripts en de
rapporttekst gehaald. De demodata is opnieuw gegenereerd zonder die kolommen.
</commit_message>
<xml_diff>
--- a/data/demo/demo_leiden_2026/config.xlsx
+++ b/data/demo/demo_leiden_2026/config.xlsx
@@ -484,7 +484,7 @@
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>Studentnummer</t>
+          <t>A_Nummer_Aanvraag</t>
         </is>
       </c>
     </row>
@@ -496,7 +496,7 @@
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>Gedragswetenschappen</t>
+          <t>Farmacie</t>
         </is>
       </c>
     </row>
@@ -532,7 +532,7 @@
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>Scores en ranking</t>
+          <t>2 Master beoordelingen</t>
         </is>
       </c>
     </row>
@@ -544,7 +544,7 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
     </row>
@@ -556,7 +556,7 @@
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>Totale selectiescore %</t>
+          <t>C_Sc_Totaal</t>
         </is>
       </c>
     </row>
@@ -571,7 +571,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D8"/>
+  <dimension ref="A1:D12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -605,153 +605,236 @@
     <row r="2">
       <c r="A2" s="4" t="inlineStr">
         <is>
-          <t>WI SCORE</t>
+          <t>A_Gem_Cijfer_Bachelor_1</t>
         </is>
       </c>
       <c r="B2" s="4" t="inlineStr">
         <is>
-          <t>Schooldiploma</t>
+          <t>Bachelordiploma</t>
         </is>
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>Wiskunde puntenscore</t>
+          <t>Gemiddeld bachelorcijfer</t>
         </is>
       </c>
       <c r="D2" s="4" t="inlineStr">
         <is>
-          <t>Vakkennis wiskunde</t>
+          <t>Studieresultaat</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t>EN SCORE</t>
+          <t>A_Score_Gem_Cijfer_Ba1</t>
         </is>
       </c>
       <c r="B3" s="4" t="inlineStr">
         <is>
-          <t>Schooldiploma</t>
+          <t>Bachelordiploma</t>
         </is>
       </c>
       <c r="C3" s="4" t="inlineStr">
         <is>
-          <t>Engels puntenscore</t>
+          <t>Puntenscore bachelorcijfer</t>
         </is>
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t>Vakkennis Engels</t>
+          <t>Studieresultaat</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>BIO SCORE</t>
+          <t>A_Bereken_Pnt_Duur_Ba</t>
         </is>
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>Schooldiploma</t>
+          <t>Bachelordiploma</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>Biologie puntenscore</t>
+          <t>Puntenscore studietempo</t>
         </is>
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>Vakkennis biologie</t>
+          <t>Studietempo</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>WI+EN+BIO (0-5)</t>
+          <t>C_B1_Sc_NL_Docs</t>
         </is>
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>Schooldiploma</t>
+          <t>Gesprek</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>Gemiddelde kernvakken (0-5)</t>
+          <t>Nederlandse documenten (B1)</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>Profielsterkheid</t>
+          <t>Taalbeheersing</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>COMBICIJF 
-SCORE</t>
+          <t>C_B2_Sc_NL_Docs</t>
         </is>
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>Schooldiploma</t>
+          <t>Gesprek</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>Combinatiecijfer puntenscore</t>
+          <t>Nederlandse documenten (B2)</t>
         </is>
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>Algemeen studieniveau</t>
+          <t>Taalbeheersing</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>Matching Score (1-3)</t>
+          <t>C_B1_Sc_NL_Gespr_Schrijf</t>
         </is>
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>Matchingsvragenlijst</t>
+          <t>Gesprek</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>Matchingscore (1-3)</t>
+          <t>Taalvaardigheid gesprek/schrijf (B1)</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>Studiemotivatie</t>
+          <t>Taalbeheersing</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>Vragenlijst %</t>
+          <t>C_B2_Sc_NL_Gespr_Schrijf</t>
         </is>
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>Deelscore</t>
+          <t>Gesprek</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>Vragenlijst score percentage</t>
-        </is>
-      </c>
-      <c r="D8" s="4" t="inlineStr"/>
+          <t>Taalvaardigheid gesprek/schrijf (B2)</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>Taalbeheersing</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>C_B1_Sc_Beoord_Gesprek</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>Gesprek</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>Gespreksbeoordeling (B1)</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>Communicatievaardigheid</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>C_B2_Sc_Beoord_Gesprek</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>Gesprek</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>Gespreksbeoordeling (B2)</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t>Communicatievaardigheid</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>C_B1_B2_Sc_SubTotaal</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>Gesprek</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>Subtotaal gesprek B1+B2</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>C_A_Sc_SubTotaal</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>Bachelordiploma</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="inlineStr">
+        <is>
+          <t>Subtotaal diploma</t>
+        </is>
+      </c>
+      <c r="D12" s="4" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Regenereer voorbeeldconfigs naar nieuw kolommen-formaat met alle kolommen
</commit_message>
<xml_diff>
--- a/data/demo/demo_leiden_2026/config.xlsx
+++ b/data/demo/demo_leiden_2026/config.xlsx
@@ -18,7 +18,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="4">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -26,39 +26,16 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
-    <font>
-      <name val="Calibri"/>
-      <b val="1"/>
-      <color rgb="00FFFFFF"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <b val="1"/>
-      <color rgb="002C3E50"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <color rgb="00333333"/>
-      <sz val="11"/>
-    </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="002C3E50"/>
-        <bgColor rgb="002C3E50"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -66,32 +43,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color rgb="00D5D8DC"/>
-      </left>
-      <right style="thin">
-        <color rgb="00D5D8DC"/>
-      </right>
-      <top style="thin">
-        <color rgb="00D5D8DC"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="00D5D8DC"/>
-      </bottom>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -457,104 +414,88 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B8"/>
+  <dimension ref="A1:B7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="25" customWidth="1" min="1" max="1"/>
-    <col width="50" customWidth="1" min="2" max="2"/>
-  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>instelling</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>waarde</t>
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>koppel_id_kolom</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>A_Nummer_Aanvraag</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>Koppel_id_kolom</t>
-        </is>
-      </c>
-      <c r="B2" s="3" t="inlineStr">
-        <is>
-          <t>A_Nummer_Aanvraag</t>
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>opleiding</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Farmacie</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>opleiding</t>
-        </is>
-      </c>
-      <c r="B3" s="3" t="inlineStr">
-        <is>
-          <t>Farmacie</t>
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>instellingscode</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Universiteit Leiden</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>instellingscode</t>
-        </is>
-      </c>
-      <c r="B4" s="3" t="inlineStr">
-        <is>
-          <t>Universiteit Leiden</t>
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>jaar</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>2026</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>jaar</t>
-        </is>
-      </c>
-      <c r="B5" s="3" t="inlineStr">
-        <is>
-          <t>2026</t>
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>blad_naam</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>2 Master beoordelingen</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>blad_naam</t>
-        </is>
-      </c>
-      <c r="B6" s="3" t="inlineStr">
-        <is>
-          <t>2 Master beoordelingen</t>
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>header_rij</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>1</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t>header_rij</t>
-        </is>
-      </c>
-      <c r="B7" s="3" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="2" t="inlineStr">
+      <c r="A7" t="inlineStr">
         <is>
           <t>totaalscore_kolom</t>
         </is>
       </c>
-      <c r="B8" s="3" t="inlineStr">
+      <c r="B7" t="inlineStr">
         <is>
           <t>C_Sc_Totaal</t>
         </is>
@@ -571,270 +512,710 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D12"/>
+  <dimension ref="A1:F40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="40" customWidth="1" min="1" max="1"/>
-    <col width="25" customWidth="1" min="2" max="2"/>
-    <col width="35" customWidth="1" min="3" max="3"/>
-    <col width="25" customWidth="1" min="4" max="4"/>
-  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>meenemen</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
         <is>
           <t>kolom_naam</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>instrument</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>item</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>criterium (optioneel)</t>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>criterium</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>schaal</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="4" t="inlineStr">
+      <c r="A2" t="b">
+        <v>0</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>A_Nummer_Aanvraag</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr"/>
+      <c r="D2" t="inlineStr"/>
+      <c r="E2" t="inlineStr"/>
+      <c r="F2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="b">
+        <v>0</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Selectie</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr"/>
+      <c r="D3" t="inlineStr"/>
+      <c r="E3" t="inlineStr"/>
+      <c r="F3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" t="b">
+        <v>0</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>A_Geslacht</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr"/>
+      <c r="D4" t="inlineStr"/>
+      <c r="E4" t="inlineStr"/>
+      <c r="F4" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="b">
+        <v>0</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>A_Gevolgde_Opleiding_1</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr"/>
+      <c r="D5" t="inlineStr"/>
+      <c r="E5" t="inlineStr"/>
+      <c r="F5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="b">
+        <v>1</v>
+      </c>
+      <c r="B6" t="inlineStr">
         <is>
           <t>A_Gem_Cijfer_Bachelor_1</t>
         </is>
       </c>
-      <c r="B2" s="4" t="inlineStr">
+      <c r="C6" t="inlineStr">
         <is>
           <t>Bachelordiploma</t>
         </is>
       </c>
-      <c r="C2" s="4" t="inlineStr">
+      <c r="D6" t="inlineStr">
         <is>
           <t>Gemiddeld bachelorcijfer</t>
         </is>
       </c>
-      <c r="D2" s="4" t="inlineStr">
+      <c r="E6" t="inlineStr">
         <is>
           <t>Studieresultaat</t>
         </is>
       </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="4" t="inlineStr">
+      <c r="F6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="b">
+        <v>1</v>
+      </c>
+      <c r="B7" t="inlineStr">
         <is>
           <t>A_Score_Gem_Cijfer_Ba1</t>
         </is>
       </c>
-      <c r="B3" s="4" t="inlineStr">
+      <c r="C7" t="inlineStr">
         <is>
           <t>Bachelordiploma</t>
         </is>
       </c>
-      <c r="C3" s="4" t="inlineStr">
+      <c r="D7" t="inlineStr">
         <is>
           <t>Puntenscore bachelorcijfer</t>
         </is>
       </c>
-      <c r="D3" s="4" t="inlineStr">
+      <c r="E7" t="inlineStr">
         <is>
           <t>Studieresultaat</t>
         </is>
       </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="4" t="inlineStr">
+      <c r="F7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="b">
+        <v>0</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>A_Bachelor_Maanden_1</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr"/>
+      <c r="D8" t="inlineStr"/>
+      <c r="E8" t="inlineStr"/>
+      <c r="F8" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" t="b">
+        <v>0</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>A_Mnd_Nominaal1</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr"/>
+      <c r="D9" t="inlineStr"/>
+      <c r="E9" t="inlineStr"/>
+      <c r="F9" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="b">
+        <v>0</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>A_Mnd_Ba_boven_Nominaal1</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr"/>
+      <c r="D10" t="inlineStr"/>
+      <c r="E10" t="inlineStr"/>
+      <c r="F10" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" t="b">
+        <v>0</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>A_Score_Duur_Ba_Nominaal1</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr"/>
+      <c r="D11" t="inlineStr"/>
+      <c r="E11" t="inlineStr"/>
+      <c r="F11" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" t="b">
+        <v>1</v>
+      </c>
+      <c r="B12" t="inlineStr">
         <is>
           <t>A_Bereken_Pnt_Duur_Ba</t>
         </is>
       </c>
-      <c r="B4" s="4" t="inlineStr">
+      <c r="C12" t="inlineStr">
         <is>
           <t>Bachelordiploma</t>
         </is>
       </c>
-      <c r="C4" s="4" t="inlineStr">
+      <c r="D12" t="inlineStr">
         <is>
           <t>Puntenscore studietempo</t>
         </is>
       </c>
-      <c r="D4" s="4" t="inlineStr">
+      <c r="E12" t="inlineStr">
         <is>
           <t>Studietempo</t>
         </is>
       </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="4" t="inlineStr">
+      <c r="F12" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" t="b">
+        <v>0</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>B1_Achternaam</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr"/>
+      <c r="D13" t="inlineStr"/>
+      <c r="E13" t="inlineStr"/>
+      <c r="F13" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" t="b">
+        <v>0</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>B1_NL_Docs</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr"/>
+      <c r="D14" t="inlineStr"/>
+      <c r="E14" t="inlineStr"/>
+      <c r="F14" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" t="b">
+        <v>0</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>B1_Score_NL_Docs</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr"/>
+      <c r="D15" t="inlineStr"/>
+      <c r="E15" t="inlineStr"/>
+      <c r="F15" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" t="b">
+        <v>0</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>B1_NL_Gespr_Schrijf</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr"/>
+      <c r="D16" t="inlineStr"/>
+      <c r="E16" t="inlineStr"/>
+      <c r="F16" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" t="b">
+        <v>0</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>B1_Score_NL_Gespr_Schrijf</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr"/>
+      <c r="D17" t="inlineStr"/>
+      <c r="E17" t="inlineStr"/>
+      <c r="F17" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" t="b">
+        <v>0</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>B1_Beoord_Gespr_Schrijfop</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr"/>
+      <c r="D18" t="inlineStr"/>
+      <c r="E18" t="inlineStr"/>
+      <c r="F18" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" t="b">
+        <v>0</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>B1_Score_Beoord_Gesprek</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr"/>
+      <c r="D19" t="inlineStr"/>
+      <c r="E19" t="inlineStr"/>
+      <c r="F19" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" t="b">
+        <v>0</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>B2_Achternaam</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr"/>
+      <c r="D20" t="inlineStr"/>
+      <c r="E20" t="inlineStr"/>
+      <c r="F20" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" t="b">
+        <v>0</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>B2_NL_Docs</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr"/>
+      <c r="D21" t="inlineStr"/>
+      <c r="E21" t="inlineStr"/>
+      <c r="F21" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" t="b">
+        <v>0</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>B2_Score_NL_Docs</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr"/>
+      <c r="D22" t="inlineStr"/>
+      <c r="E22" t="inlineStr"/>
+      <c r="F22" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" t="b">
+        <v>0</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>B2_NL_Gespr_Schrijf</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr"/>
+      <c r="D23" t="inlineStr"/>
+      <c r="E23" t="inlineStr"/>
+      <c r="F23" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" t="b">
+        <v>0</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>B2_Score_NL_Gespr_Schrijf</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr"/>
+      <c r="D24" t="inlineStr"/>
+      <c r="E24" t="inlineStr"/>
+      <c r="F24" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" t="b">
+        <v>0</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>B2_Beoord_Gespr_Schrijfop</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr"/>
+      <c r="D25" t="inlineStr"/>
+      <c r="E25" t="inlineStr"/>
+      <c r="F25" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" t="b">
+        <v>0</v>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>B2_Score_Beoord_Gesprek</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr"/>
+      <c r="D26" t="inlineStr"/>
+      <c r="E26" t="inlineStr"/>
+      <c r="F26" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" t="b">
+        <v>0</v>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>C_Sc_Gem_Cijfer_Ba</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr"/>
+      <c r="D27" t="inlineStr"/>
+      <c r="E27" t="inlineStr"/>
+      <c r="F27" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" t="b">
+        <v>0</v>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>C_Sc_Duur_Ba_Nominaal1</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr"/>
+      <c r="D28" t="inlineStr"/>
+      <c r="E28" t="inlineStr"/>
+      <c r="F28" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" t="b">
+        <v>1</v>
+      </c>
+      <c r="B29" t="inlineStr">
         <is>
           <t>C_B1_Sc_NL_Docs</t>
         </is>
       </c>
-      <c r="B5" s="4" t="inlineStr">
+      <c r="C29" t="inlineStr">
         <is>
           <t>Gesprek</t>
         </is>
       </c>
-      <c r="C5" s="4" t="inlineStr">
+      <c r="D29" t="inlineStr">
         <is>
           <t>Nederlandse documenten (B1)</t>
         </is>
       </c>
-      <c r="D5" s="4" t="inlineStr">
+      <c r="E29" t="inlineStr">
         <is>
           <t>Taalbeheersing</t>
         </is>
       </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="4" t="inlineStr">
+      <c r="F29" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" t="b">
+        <v>1</v>
+      </c>
+      <c r="B30" t="inlineStr">
         <is>
           <t>C_B2_Sc_NL_Docs</t>
         </is>
       </c>
-      <c r="B6" s="4" t="inlineStr">
+      <c r="C30" t="inlineStr">
         <is>
           <t>Gesprek</t>
         </is>
       </c>
-      <c r="C6" s="4" t="inlineStr">
+      <c r="D30" t="inlineStr">
         <is>
           <t>Nederlandse documenten (B2)</t>
         </is>
       </c>
-      <c r="D6" s="4" t="inlineStr">
+      <c r="E30" t="inlineStr">
         <is>
           <t>Taalbeheersing</t>
         </is>
       </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="4" t="inlineStr">
+      <c r="F30" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" t="b">
+        <v>1</v>
+      </c>
+      <c r="B31" t="inlineStr">
         <is>
           <t>C_B1_Sc_NL_Gespr_Schrijf</t>
         </is>
       </c>
-      <c r="B7" s="4" t="inlineStr">
+      <c r="C31" t="inlineStr">
         <is>
           <t>Gesprek</t>
         </is>
       </c>
-      <c r="C7" s="4" t="inlineStr">
+      <c r="D31" t="inlineStr">
         <is>
           <t>Taalvaardigheid gesprek/schrijf (B1)</t>
         </is>
       </c>
-      <c r="D7" s="4" t="inlineStr">
+      <c r="E31" t="inlineStr">
         <is>
           <t>Taalbeheersing</t>
         </is>
       </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="4" t="inlineStr">
+      <c r="F31" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" t="b">
+        <v>1</v>
+      </c>
+      <c r="B32" t="inlineStr">
         <is>
           <t>C_B2_Sc_NL_Gespr_Schrijf</t>
         </is>
       </c>
-      <c r="B8" s="4" t="inlineStr">
+      <c r="C32" t="inlineStr">
         <is>
           <t>Gesprek</t>
         </is>
       </c>
-      <c r="C8" s="4" t="inlineStr">
+      <c r="D32" t="inlineStr">
         <is>
           <t>Taalvaardigheid gesprek/schrijf (B2)</t>
         </is>
       </c>
-      <c r="D8" s="4" t="inlineStr">
+      <c r="E32" t="inlineStr">
         <is>
           <t>Taalbeheersing</t>
         </is>
       </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="4" t="inlineStr">
+      <c r="F32" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" t="b">
+        <v>1</v>
+      </c>
+      <c r="B33" t="inlineStr">
         <is>
           <t>C_B1_Sc_Beoord_Gesprek</t>
         </is>
       </c>
-      <c r="B9" s="4" t="inlineStr">
+      <c r="C33" t="inlineStr">
         <is>
           <t>Gesprek</t>
         </is>
       </c>
-      <c r="C9" s="4" t="inlineStr">
+      <c r="D33" t="inlineStr">
         <is>
           <t>Gespreksbeoordeling (B1)</t>
         </is>
       </c>
-      <c r="D9" s="4" t="inlineStr">
+      <c r="E33" t="inlineStr">
         <is>
           <t>Communicatievaardigheid</t>
         </is>
       </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="4" t="inlineStr">
+      <c r="F33" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" t="b">
+        <v>1</v>
+      </c>
+      <c r="B34" t="inlineStr">
         <is>
           <t>C_B2_Sc_Beoord_Gesprek</t>
         </is>
       </c>
-      <c r="B10" s="4" t="inlineStr">
+      <c r="C34" t="inlineStr">
         <is>
           <t>Gesprek</t>
         </is>
       </c>
-      <c r="C10" s="4" t="inlineStr">
+      <c r="D34" t="inlineStr">
         <is>
           <t>Gespreksbeoordeling (B2)</t>
         </is>
       </c>
-      <c r="D10" s="4" t="inlineStr">
+      <c r="E34" t="inlineStr">
         <is>
           <t>Communicatievaardigheid</t>
         </is>
       </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="4" t="inlineStr">
+      <c r="F34" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" t="b">
+        <v>0</v>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>C_B1_Sc_SubTotaal</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr"/>
+      <c r="D35" t="inlineStr"/>
+      <c r="E35" t="inlineStr"/>
+      <c r="F35" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" t="b">
+        <v>0</v>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>C_B2_Sc_SubTotaal</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr"/>
+      <c r="D36" t="inlineStr"/>
+      <c r="E36" t="inlineStr"/>
+      <c r="F36" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" t="b">
+        <v>1</v>
+      </c>
+      <c r="B37" t="inlineStr">
         <is>
           <t>C_B1_B2_Sc_SubTotaal</t>
         </is>
       </c>
-      <c r="B11" s="4" t="inlineStr">
+      <c r="C37" t="inlineStr">
         <is>
           <t>Gesprek</t>
         </is>
       </c>
-      <c r="C11" s="4" t="inlineStr">
+      <c r="D37" t="inlineStr">
         <is>
           <t>Subtotaal gesprek B1+B2</t>
         </is>
       </c>
-      <c r="D11" s="4" t="inlineStr"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="4" t="inlineStr">
+      <c r="E37" t="inlineStr"/>
+      <c r="F37" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" t="b">
+        <v>1</v>
+      </c>
+      <c r="B38" t="inlineStr">
         <is>
           <t>C_A_Sc_SubTotaal</t>
         </is>
       </c>
-      <c r="B12" s="4" t="inlineStr">
+      <c r="C38" t="inlineStr">
         <is>
           <t>Bachelordiploma</t>
         </is>
       </c>
-      <c r="C12" s="4" t="inlineStr">
+      <c r="D38" t="inlineStr">
         <is>
           <t>Subtotaal diploma</t>
         </is>
       </c>
-      <c r="D12" s="4" t="inlineStr"/>
+      <c r="E38" t="inlineStr"/>
+      <c r="F38" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" t="b">
+        <v>0</v>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>C_Sc_Totaal</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr"/>
+      <c r="D39" t="inlineStr"/>
+      <c r="E39" t="inlineStr"/>
+      <c r="F39" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" t="b">
+        <v>0</v>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Rangnummer definitief</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr"/>
+      <c r="D40" t="inlineStr"/>
+      <c r="E40" t="inlineStr"/>
+      <c r="F40" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>